<commit_message>
Fix the backend and frontend issues , export issues
</commit_message>
<xml_diff>
--- a/backend/exports/single_student_teams.xlsx
+++ b/backend/exports/single_student_teams.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
   <si>
     <t>Team ID</t>
   </si>
@@ -31,46 +31,25 @@
     <t>Current Review</t>
   </si>
   <si>
-    <t>BTECH-IT-063</t>
+    <t>Abstract</t>
+  </si>
+  <si>
+    <t>BTECH-IT-148</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>MOHAMMED IMRAN N</t>
-  </si>
-  <si>
-    <t>43120126</t>
-  </si>
-  <si>
-    <t>Ms. Arthi D</t>
+    <t>SHRADDHA</t>
+  </si>
+  <si>
+    <t>43120305</t>
+  </si>
+  <si>
+    <t>Dr. C. Geetha</t>
   </si>
   <si>
     <t>Zeroth Review</t>
-  </si>
-  <si>
-    <t>BTECH-IT-084</t>
-  </si>
-  <si>
-    <t>PRISIL JESIN M</t>
-  </si>
-  <si>
-    <t>43120160</t>
-  </si>
-  <si>
-    <t>Dr. P. Jeyanthi</t>
-  </si>
-  <si>
-    <t>BTECH-IT-149</t>
-  </si>
-  <si>
-    <t>SHRADDHA</t>
-  </si>
-  <si>
-    <t>43120305</t>
-  </si>
-  <si>
-    <t>Dr. C. Geetha</t>
   </si>
 </sst>
 </file>
@@ -447,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -456,9 +435,10 @@
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -477,8 +457,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -497,65 +480,31 @@
       <c r="F2" t="s">
         <v>5</v>
       </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>